<commit_message>
feat: actualiser le corpus Mosar et les statistiques de 193 revues
</commit_message>
<xml_diff>
--- a/tests/fixtures/minimal-corpus.xlsx
+++ b/tests/fixtures/minimal-corpus.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Éditeur public</t>
+          <t>éditeur public</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Association</t>
+          <t>association</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Éditeur privé</t>
+          <t>éditeur privé</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Organisme de recherche public</t>
+          <t>organisme de recherche public</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Coédition public/privé</t>
+          <t>coédition public/privé</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Coédition privé/Association</t>
+          <t>coédition privé/association</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Éditeur public</t>
+          <t>éditeur public</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Association</t>
+          <t>association</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Éditeur privé</t>
+          <t>éditeur privé</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Organisme de recherche public</t>
+          <t>organisme de recherche public</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Coédition public/privé</t>
+          <t>coédition public/privé</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Coédition privé/Association</t>
+          <t>coédition privé/association</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">

</xml_diff>